<commit_message>
Updated NZL_grids model - 2025-09-07 17:33
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL_grids/SuppXLS/Scen_Base_VS.xlsx
+++ b/VerveStacks_NZL_grids/SuppXLS/Scen_Base_VS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NZL_grids\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{64FBBCA5-F987-4B3B-8926-AFDC49A01FA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C5BA3263-0157-4417-BDF4-22FAF6EEEEB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2047,7 +2047,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01C1EA7A-3DD2-4EFB-857F-EC304B5960BC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99657A21-416A-4E9C-AC4B-4F5BF50882F1}">
   <dimension ref="B2:AE183"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated NZL_grids model - 2025-09-09 08:36
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL_grids/SuppXLS/Scen_Base_VS.xlsx
+++ b/VerveStacks_NZL_grids/SuppXLS/Scen_Base_VS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NZL_grids\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D717F03B-5BEF-4A91-BDD9-42CA8A029183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{65BD5AD4-2B0D-426A-840A-0F57E7E326E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2047,7 +2047,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB03C1DC-4E3D-4776-96E6-29AB18FFFE42}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B73037B3-4B95-418B-8B5E-21D8D209B97F}">
   <dimension ref="B2:AE183"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated NZL_grids model - 2025-09-09 08:40
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL_grids/SuppXLS/Scen_Base_VS.xlsx
+++ b/VerveStacks_NZL_grids/SuppXLS/Scen_Base_VS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NZL_grids\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{65BD5AD4-2B0D-426A-840A-0F57E7E326E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BC537E01-0841-44F6-846B-0CA96150F85C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2047,7 +2047,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B73037B3-4B95-418B-8B5E-21D8D209B97F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD3A70BB-1D85-49E4-ACE4-89398CABFDAF}">
   <dimension ref="B2:AE183"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>